<commit_message>
Auto update RUP 2026-06-30 10:03:02
</commit_message>
<xml_diff>
--- a/output/rup/2026/Rekap RUP Tahun 2026 (2026-06-30).xlsx
+++ b/output/rup/2026/Rekap RUP Tahun 2026 (2026-06-30).xlsx
@@ -505,19 +505,19 @@
         <v>1581202807</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>486896807</v>
+        <v>0</v>
       </c>
       <c r="E2" s="3" t="n">
         <v>1094306000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>1581202807</v>
+        <v>1094306000</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>0</v>
+        <v>-486896807</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>100</v>
+        <v>69.20718804415834</v>
       </c>
     </row>
     <row r="3">
@@ -533,19 +533,19 @@
         <v>830740630</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>830740630</v>
+        <v>0</v>
       </c>
       <c r="E3" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>830740630</v>
+        <v>0</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>0</v>
+        <v>-830740630</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -561,19 +561,19 @@
         <v>1385846979</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>1385846979</v>
+        <v>0</v>
       </c>
       <c r="E4" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>1385846979</v>
+        <v>0</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>0</v>
+        <v>-1385846979</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -589,19 +589,19 @@
         <v>1363592000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>1363592000</v>
+        <v>0</v>
       </c>
       <c r="E5" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>1363592000</v>
+        <v>0</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>0</v>
+        <v>-1363592000</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -617,19 +617,19 @@
         <v>3636937261</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>2417247421</v>
+        <v>0</v>
       </c>
       <c r="E6" s="3" t="n">
         <v>1219689840</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>3636937261</v>
+        <v>1219689840</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>0</v>
+        <v>-2417247421</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>100</v>
+        <v>33.53618037569991</v>
       </c>
     </row>
     <row r="7">
@@ -645,19 +645,19 @@
         <v>1145858598</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>1145858598</v>
+        <v>0</v>
       </c>
       <c r="E7" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>1145858598</v>
+        <v>0</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>0</v>
+        <v>-1145858598</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -729,19 +729,19 @@
         <v>2454000424</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>2454000424</v>
+        <v>0</v>
       </c>
       <c r="E10" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>2454000424</v>
+        <v>0</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>0</v>
+        <v>-2454000424</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -757,19 +757,19 @@
         <v>978184643</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>978184643</v>
+        <v>0</v>
       </c>
       <c r="E11" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>978184643</v>
+        <v>0</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>0</v>
+        <v>-978184643</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -785,19 +785,19 @@
         <v>4891035773</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>4891035773</v>
+        <v>0</v>
       </c>
       <c r="E12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>4891035773</v>
+        <v>0</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>0</v>
+        <v>-4891035773</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -813,19 +813,19 @@
         <v>4363300381</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>4363300381</v>
+        <v>0</v>
       </c>
       <c r="E13" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>4363300381</v>
+        <v>0</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>0</v>
+        <v>-4363300381</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -841,19 +841,19 @@
         <v>15288269163</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>15288269163</v>
+        <v>0</v>
       </c>
       <c r="E14" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>15288269163</v>
+        <v>0</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>0</v>
+        <v>-15288269163</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -869,19 +869,19 @@
         <v>2474291200</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>2474291200</v>
+        <v>0</v>
       </c>
       <c r="E15" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>2474291200</v>
+        <v>0</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>0</v>
+        <v>-2474291200</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -897,19 +897,19 @@
         <v>105032048100</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>104997048100</v>
+        <v>0</v>
       </c>
       <c r="E16" s="3" t="n">
         <v>35000000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>105032048100</v>
+        <v>35000000</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>0</v>
+        <v>-104997048100</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>100</v>
+        <v>0.0333231624376941</v>
       </c>
     </row>
     <row r="17">
@@ -925,19 +925,19 @@
         <v>2187676345</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>2187676345</v>
+        <v>0</v>
       </c>
       <c r="E17" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>2187676345</v>
+        <v>0</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>0</v>
+        <v>-2187676345</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -953,19 +953,19 @@
         <v>1662695697</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>1662695697</v>
+        <v>0</v>
       </c>
       <c r="E18" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>1662695697</v>
+        <v>0</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>0</v>
+        <v>-1662695697</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -981,19 +981,19 @@
         <v>2181147677</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>2181147677</v>
+        <v>0</v>
       </c>
       <c r="E19" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>2181147677</v>
+        <v>0</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>0</v>
+        <v>-2181147677</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -1009,19 +1009,19 @@
         <v>575172642</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>575172642</v>
+        <v>0</v>
       </c>
       <c r="E20" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>575172642</v>
+        <v>0</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>0</v>
+        <v>-575172642</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -1037,19 +1037,19 @@
         <v>61655471600</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>9467977800</v>
+        <v>0</v>
       </c>
       <c r="E21" s="3" t="n">
         <v>52187493800</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>61655471600</v>
+        <v>52187493800</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>0</v>
+        <v>-9467977800</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>100</v>
+        <v>84.64373468517918</v>
       </c>
     </row>
     <row r="22">
@@ -1065,19 +1065,19 @@
         <v>10654182000</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>10654182000</v>
+        <v>0</v>
       </c>
       <c r="E22" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>10654182000</v>
+        <v>0</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>0</v>
+        <v>-10654182000</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -1093,19 +1093,19 @@
         <v>8063419229</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>8063419229</v>
+        <v>0</v>
       </c>
       <c r="E23" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>8063419229</v>
+        <v>0</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>0</v>
+        <v>-8063419229</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -1121,19 +1121,19 @@
         <v>11668621099</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>11668621099</v>
+        <v>0</v>
       </c>
       <c r="E24" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>11668621099</v>
+        <v>0</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>0</v>
+        <v>-11668621099</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -1149,19 +1149,19 @@
         <v>532966503</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>532966503</v>
+        <v>0</v>
       </c>
       <c r="E25" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>532966503</v>
+        <v>0</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>0</v>
+        <v>-532966503</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -1177,19 +1177,19 @@
         <v>12076302500</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>11831302500</v>
+        <v>0</v>
       </c>
       <c r="E26" s="3" t="n">
         <v>245000000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>12076302500</v>
+        <v>245000000</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>0</v>
+        <v>-11831302500</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>100</v>
+        <v>2.028766669268181</v>
       </c>
     </row>
     <row r="27">
@@ -1205,19 +1205,19 @@
         <v>28552934680</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>28552934680</v>
+        <v>0</v>
       </c>
       <c r="E27" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>28552934680</v>
+        <v>0</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>0</v>
+        <v>-28552934680</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -1233,19 +1233,19 @@
         <v>1858317230</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>1858317230</v>
+        <v>0</v>
       </c>
       <c r="E28" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>1858317230</v>
+        <v>0</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>0</v>
+        <v>-1858317230</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -1261,19 +1261,19 @@
         <v>1417613763</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>1417613763</v>
+        <v>0</v>
       </c>
       <c r="E29" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>1417613763</v>
+        <v>0</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>0</v>
+        <v>-1417613763</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -1289,19 +1289,19 @@
         <v>1292926000</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>1292926000</v>
+        <v>0</v>
       </c>
       <c r="E30" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>1292926000</v>
+        <v>0</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>0</v>
+        <v>-1292926000</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -1317,19 +1317,19 @@
         <v>5257374241</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>5051110241</v>
+        <v>0</v>
       </c>
       <c r="E31" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>5051110241</v>
+        <v>0</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>-206264000</v>
+        <v>-5257374241</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>96.07667267832227</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -1345,19 +1345,19 @@
         <v>4701405808</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>4606645808</v>
+        <v>0</v>
       </c>
       <c r="E32" s="3" t="n">
         <v>94760000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>4701405808</v>
+        <v>94760000</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>0</v>
+        <v>-4606645808</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>100</v>
+        <v>2.015567340278404</v>
       </c>
     </row>
     <row r="33">
@@ -1373,19 +1373,19 @@
         <v>465249566</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>465249566</v>
+        <v>0</v>
       </c>
       <c r="E33" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>465249566</v>
+        <v>0</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>0</v>
+        <v>-465249566</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -1401,19 +1401,19 @@
         <v>948269958</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>507369966</v>
+        <v>0</v>
       </c>
       <c r="E34" s="3" t="n">
         <v>440899992</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>948269958</v>
+        <v>440899992</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>0</v>
+        <v>-507369966</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>100</v>
+        <v>46.49519773144601</v>
       </c>
     </row>
     <row r="35">
@@ -1429,19 +1429,19 @@
         <v>943247000</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>774999698</v>
+        <v>0</v>
       </c>
       <c r="E35" s="3" t="n">
         <v>168247302</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>943247000</v>
+        <v>168247302</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>0</v>
+        <v>-774999698</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>100</v>
+        <v>17.83703547427132</v>
       </c>
     </row>
     <row r="36">
@@ -1457,19 +1457,19 @@
         <v>312595476</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>312595476</v>
+        <v>0</v>
       </c>
       <c r="E36" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>312595476</v>
+        <v>0</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>0</v>
+        <v>-312595476</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -1485,19 +1485,19 @@
         <v>219851775</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>219851775</v>
+        <v>0</v>
       </c>
       <c r="E37" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>219851775</v>
+        <v>0</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>0</v>
+        <v>-219851775</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
@@ -1905,19 +1905,19 @@
         <v>2405886712</v>
       </c>
       <c r="D52" s="3" t="n">
-        <v>2374286712</v>
+        <v>0</v>
       </c>
       <c r="E52" s="3" t="n">
         <v>31600000</v>
       </c>
       <c r="F52" s="3" t="n">
-        <v>2405886712</v>
+        <v>31600000</v>
       </c>
       <c r="G52" s="3" t="n">
-        <v>0</v>
+        <v>-2374286712</v>
       </c>
       <c r="H52" s="4" t="n">
-        <v>100</v>
+        <v>1.313445053018772</v>
       </c>
     </row>
     <row r="53">
@@ -2045,19 +2045,19 @@
         <v>1801912000</v>
       </c>
       <c r="D57" s="3" t="n">
-        <v>1780912000</v>
+        <v>0</v>
       </c>
       <c r="E57" s="3" t="n">
         <v>21000000</v>
       </c>
       <c r="F57" s="3" t="n">
-        <v>1801912000</v>
+        <v>21000000</v>
       </c>
       <c r="G57" s="3" t="n">
-        <v>0</v>
+        <v>-1780912000</v>
       </c>
       <c r="H57" s="4" t="n">
-        <v>100</v>
+        <v>1.165428722379339</v>
       </c>
     </row>
     <row r="58">
@@ -2073,19 +2073,19 @@
         <v>1367075285</v>
       </c>
       <c r="D58" s="3" t="n">
-        <v>721339185</v>
+        <v>0</v>
       </c>
       <c r="E58" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F58" s="3" t="n">
-        <v>721339185</v>
+        <v>0</v>
       </c>
       <c r="G58" s="3" t="n">
-        <v>-645736100</v>
+        <v>-1367075285</v>
       </c>
       <c r="H58" s="4" t="n">
-        <v>52.76513977794573</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59">
@@ -2101,19 +2101,19 @@
         <v>338454320</v>
       </c>
       <c r="D59" s="3" t="n">
-        <v>338454320</v>
+        <v>0</v>
       </c>
       <c r="E59" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F59" s="3" t="n">
-        <v>338454320</v>
+        <v>0</v>
       </c>
       <c r="G59" s="3" t="n">
-        <v>0</v>
+        <v>-338454320</v>
       </c>
       <c r="H59" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60">
@@ -2129,19 +2129,19 @@
         <v>887410440</v>
       </c>
       <c r="D60" s="3" t="n">
-        <v>887410440</v>
+        <v>0</v>
       </c>
       <c r="E60" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F60" s="3" t="n">
-        <v>887410440</v>
+        <v>0</v>
       </c>
       <c r="G60" s="3" t="n">
-        <v>0</v>
+        <v>-887410440</v>
       </c>
       <c r="H60" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61">
@@ -2157,19 +2157,19 @@
         <v>1424797850</v>
       </c>
       <c r="D61" s="3" t="n">
-        <v>212772837</v>
+        <v>0</v>
       </c>
       <c r="E61" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F61" s="3" t="n">
-        <v>212772837</v>
+        <v>0</v>
       </c>
       <c r="G61" s="3" t="n">
-        <v>-1212025013</v>
+        <v>-1424797850</v>
       </c>
       <c r="H61" s="4" t="n">
-        <v>14.93354562543732</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62">
@@ -2185,19 +2185,19 @@
         <v>1117262389</v>
       </c>
       <c r="D62" s="3" t="n">
-        <v>1116362329</v>
+        <v>0</v>
       </c>
       <c r="E62" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F62" s="3" t="n">
-        <v>1116362329</v>
+        <v>0</v>
       </c>
       <c r="G62" s="3" t="n">
-        <v>-900060</v>
+        <v>-1117262389</v>
       </c>
       <c r="H62" s="4" t="n">
-        <v>99.91944058899132</v>
+        <v>0</v>
       </c>
     </row>
     <row r="63">
@@ -2213,19 +2213,19 @@
         <v>509262312</v>
       </c>
       <c r="D63" s="3" t="n">
-        <v>509262312</v>
+        <v>0</v>
       </c>
       <c r="E63" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F63" s="3" t="n">
-        <v>509262312</v>
+        <v>0</v>
       </c>
       <c r="G63" s="3" t="n">
-        <v>0</v>
+        <v>-509262312</v>
       </c>
       <c r="H63" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64">
@@ -2241,19 +2241,19 @@
         <v>373421530</v>
       </c>
       <c r="D64" s="3" t="n">
-        <v>373421530</v>
+        <v>0</v>
       </c>
       <c r="E64" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F64" s="3" t="n">
-        <v>373421530</v>
+        <v>0</v>
       </c>
       <c r="G64" s="3" t="n">
-        <v>0</v>
+        <v>-373421530</v>
       </c>
       <c r="H64" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65">
@@ -2269,19 +2269,19 @@
         <v>552591787</v>
       </c>
       <c r="D65" s="3" t="n">
-        <v>552591787</v>
+        <v>0</v>
       </c>
       <c r="E65" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F65" s="3" t="n">
-        <v>552591787</v>
+        <v>0</v>
       </c>
       <c r="G65" s="3" t="n">
-        <v>0</v>
+        <v>-552591787</v>
       </c>
       <c r="H65" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66">
@@ -2297,19 +2297,19 @@
         <v>735655752</v>
       </c>
       <c r="D66" s="3" t="n">
-        <v>541055752</v>
+        <v>0</v>
       </c>
       <c r="E66" s="3" t="n">
         <v>194600000</v>
       </c>
       <c r="F66" s="3" t="n">
-        <v>735655752</v>
+        <v>194600000</v>
       </c>
       <c r="G66" s="3" t="n">
-        <v>0</v>
+        <v>-541055752</v>
       </c>
       <c r="H66" s="4" t="n">
-        <v>100</v>
+        <v>26.45259001522767</v>
       </c>
     </row>
     <row r="67">
@@ -2325,19 +2325,19 @@
         <v>289499767</v>
       </c>
       <c r="D67" s="3" t="n">
-        <v>289499767</v>
+        <v>0</v>
       </c>
       <c r="E67" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F67" s="3" t="n">
-        <v>289499767</v>
+        <v>0</v>
       </c>
       <c r="G67" s="3" t="n">
-        <v>0</v>
+        <v>-289499767</v>
       </c>
       <c r="H67" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="68">
@@ -2353,19 +2353,19 @@
         <v>429267455</v>
       </c>
       <c r="D68" s="3" t="n">
-        <v>429267455</v>
+        <v>0</v>
       </c>
       <c r="E68" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F68" s="3" t="n">
-        <v>429267455</v>
+        <v>0</v>
       </c>
       <c r="G68" s="3" t="n">
-        <v>0</v>
+        <v>-429267455</v>
       </c>
       <c r="H68" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="69">
@@ -2381,19 +2381,19 @@
         <v>153251633</v>
       </c>
       <c r="D69" s="3" t="n">
-        <v>153251633</v>
+        <v>0</v>
       </c>
       <c r="E69" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F69" s="3" t="n">
-        <v>153251633</v>
+        <v>0</v>
       </c>
       <c r="G69" s="3" t="n">
-        <v>0</v>
+        <v>-153251633</v>
       </c>
       <c r="H69" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70">
@@ -2409,19 +2409,19 @@
         <v>329330796</v>
       </c>
       <c r="D70" s="3" t="n">
-        <v>329330796</v>
+        <v>0</v>
       </c>
       <c r="E70" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F70" s="3" t="n">
-        <v>329330796</v>
+        <v>0</v>
       </c>
       <c r="G70" s="3" t="n">
-        <v>0</v>
+        <v>-329330796</v>
       </c>
       <c r="H70" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71">
@@ -2437,19 +2437,19 @@
         <v>270659900</v>
       </c>
       <c r="D71" s="3" t="n">
-        <v>270659900</v>
+        <v>0</v>
       </c>
       <c r="E71" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F71" s="3" t="n">
-        <v>270659900</v>
+        <v>0</v>
       </c>
       <c r="G71" s="3" t="n">
-        <v>0</v>
+        <v>-270659900</v>
       </c>
       <c r="H71" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72">
@@ -2465,19 +2465,19 @@
         <v>654395500</v>
       </c>
       <c r="D72" s="3" t="n">
-        <v>654395500</v>
+        <v>0</v>
       </c>
       <c r="E72" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F72" s="3" t="n">
-        <v>654395500</v>
+        <v>0</v>
       </c>
       <c r="G72" s="3" t="n">
-        <v>0</v>
+        <v>-654395500</v>
       </c>
       <c r="H72" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73">
@@ -2493,19 +2493,19 @@
         <v>448879549</v>
       </c>
       <c r="D73" s="3" t="n">
-        <v>448879549</v>
+        <v>0</v>
       </c>
       <c r="E73" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F73" s="3" t="n">
-        <v>448879549</v>
+        <v>0</v>
       </c>
       <c r="G73" s="3" t="n">
-        <v>0</v>
+        <v>-448879549</v>
       </c>
       <c r="H73" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74">
@@ -2521,19 +2521,19 @@
         <v>1291889268</v>
       </c>
       <c r="D74" s="3" t="n">
-        <v>350390301</v>
+        <v>0</v>
       </c>
       <c r="E74" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F74" s="3" t="n">
-        <v>350390301</v>
+        <v>0</v>
       </c>
       <c r="G74" s="3" t="n">
-        <v>-941498967</v>
+        <v>-1291889268</v>
       </c>
       <c r="H74" s="4" t="n">
-        <v>27.12231687956092</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75">
@@ -2577,19 +2577,19 @@
         <v>992988041</v>
       </c>
       <c r="D76" s="3" t="n">
-        <v>992988041</v>
+        <v>0</v>
       </c>
       <c r="E76" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F76" s="3" t="n">
-        <v>992988041</v>
+        <v>0</v>
       </c>
       <c r="G76" s="3" t="n">
-        <v>0</v>
+        <v>-992988041</v>
       </c>
       <c r="H76" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="77">
@@ -2605,19 +2605,19 @@
         <v>85061928740</v>
       </c>
       <c r="D77" s="3" t="n">
-        <v>85061928740</v>
+        <v>0</v>
       </c>
       <c r="E77" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F77" s="3" t="n">
-        <v>85061928740</v>
+        <v>0</v>
       </c>
       <c r="G77" s="3" t="n">
-        <v>0</v>
+        <v>-85061928740</v>
       </c>
       <c r="H77" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="78">
@@ -2633,19 +2633,19 @@
         <v>1028700867</v>
       </c>
       <c r="D78" s="3" t="n">
-        <v>1028700867</v>
+        <v>0</v>
       </c>
       <c r="E78" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F78" s="3" t="n">
-        <v>1028700867</v>
+        <v>0</v>
       </c>
       <c r="G78" s="3" t="n">
-        <v>0</v>
+        <v>-1028700867</v>
       </c>
       <c r="H78" s="4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="79">
@@ -2661,19 +2661,19 @@
         <v>8905641688</v>
       </c>
       <c r="D79" s="3" t="n">
-        <v>8755641688</v>
+        <v>0</v>
       </c>
       <c r="E79" s="3" t="n">
         <v>150000000</v>
       </c>
       <c r="F79" s="3" t="n">
-        <v>8905641688</v>
+        <v>150000000</v>
       </c>
       <c r="G79" s="3" t="n">
-        <v>0</v>
+        <v>-8755641688</v>
       </c>
       <c r="H79" s="4" t="n">
-        <v>100</v>
+        <v>1.684325568612524</v>
       </c>
     </row>
     <row r="80">
@@ -2689,19 +2689,19 @@
         <v>11974816559</v>
       </c>
       <c r="D80" s="3" t="n">
-        <v>11799027759</v>
+        <v>0</v>
       </c>
       <c r="E80" s="3" t="n">
         <v>175788800</v>
       </c>
       <c r="F80" s="3" t="n">
-        <v>11974816559</v>
+        <v>175788800</v>
       </c>
       <c r="G80" s="3" t="n">
-        <v>0</v>
+        <v>-11799027759</v>
       </c>
       <c r="H80" s="4" t="n">
-        <v>100</v>
+        <v>1.467987414536894</v>
       </c>
     </row>
     <row r="81">

</xml_diff>

<commit_message>
Auto update RUP 2026-06-30 10:08:52
</commit_message>
<xml_diff>
--- a/output/rup/2026/Rekap RUP Tahun 2026 (2026-06-30).xlsx
+++ b/output/rup/2026/Rekap RUP Tahun 2026 (2026-06-30).xlsx
@@ -505,19 +505,19 @@
         <v>1581202807</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0</v>
+        <v>486896807</v>
       </c>
       <c r="E2" s="3" t="n">
         <v>1094306000</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>1094306000</v>
+        <v>1581202807</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>-486896807</v>
+        <v>0</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>69.20718804415834</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3">
@@ -533,19 +533,19 @@
         <v>830740630</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>0</v>
+        <v>830740630</v>
       </c>
       <c r="E3" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>0</v>
+        <v>830740630</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>-830740630</v>
+        <v>0</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4">
@@ -561,19 +561,19 @@
         <v>1385846979</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>0</v>
+        <v>1385846979</v>
       </c>
       <c r="E4" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>0</v>
+        <v>1385846979</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>-1385846979</v>
+        <v>0</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5">
@@ -589,19 +589,19 @@
         <v>1363592000</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>0</v>
+        <v>1363592000</v>
       </c>
       <c r="E5" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>0</v>
+        <v>1363592000</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>-1363592000</v>
+        <v>0</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6">
@@ -617,19 +617,19 @@
         <v>3636937261</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>0</v>
+        <v>2417247421</v>
       </c>
       <c r="E6" s="3" t="n">
         <v>1219689840</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>1219689840</v>
+        <v>3636937261</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>-2417247421</v>
+        <v>0</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>33.53618037569991</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7">
@@ -645,19 +645,19 @@
         <v>1145858598</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>0</v>
+        <v>1145858598</v>
       </c>
       <c r="E7" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>0</v>
+        <v>1145858598</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>-1145858598</v>
+        <v>0</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8">
@@ -729,19 +729,19 @@
         <v>2454000424</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>0</v>
+        <v>2454000424</v>
       </c>
       <c r="E10" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>0</v>
+        <v>2454000424</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>-2454000424</v>
+        <v>0</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11">
@@ -757,19 +757,19 @@
         <v>978184643</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>0</v>
+        <v>978184643</v>
       </c>
       <c r="E11" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0</v>
+        <v>978184643</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>-978184643</v>
+        <v>0</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12">
@@ -785,19 +785,19 @@
         <v>4891035773</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>0</v>
+        <v>4891035773</v>
       </c>
       <c r="E12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0</v>
+        <v>4891035773</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>-4891035773</v>
+        <v>0</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13">
@@ -813,19 +813,19 @@
         <v>4363300381</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>0</v>
+        <v>4363300381</v>
       </c>
       <c r="E13" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0</v>
+        <v>4363300381</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>-4363300381</v>
+        <v>0</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14">
@@ -841,19 +841,19 @@
         <v>15288269163</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>0</v>
+        <v>15288269163</v>
       </c>
       <c r="E14" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0</v>
+        <v>15288269163</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>-15288269163</v>
+        <v>0</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15">
@@ -869,19 +869,19 @@
         <v>2474291200</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>0</v>
+        <v>2474291200</v>
       </c>
       <c r="E15" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0</v>
+        <v>2474291200</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>-2474291200</v>
+        <v>0</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16">
@@ -897,19 +897,19 @@
         <v>105032048100</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>0</v>
+        <v>104997048100</v>
       </c>
       <c r="E16" s="3" t="n">
         <v>35000000</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>35000000</v>
+        <v>105032048100</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>-104997048100</v>
+        <v>0</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>0.0333231624376941</v>
+        <v>100</v>
       </c>
     </row>
     <row r="17">
@@ -925,19 +925,19 @@
         <v>2187676345</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>0</v>
+        <v>2187676345</v>
       </c>
       <c r="E17" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>0</v>
+        <v>2187676345</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>-2187676345</v>
+        <v>0</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="18">
@@ -953,19 +953,19 @@
         <v>1662695697</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>0</v>
+        <v>1662695697</v>
       </c>
       <c r="E18" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>0</v>
+        <v>1662695697</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>-1662695697</v>
+        <v>0</v>
       </c>
       <c r="H18" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="19">
@@ -981,19 +981,19 @@
         <v>2181147677</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>0</v>
+        <v>2181147677</v>
       </c>
       <c r="E19" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>0</v>
+        <v>2181147677</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>-2181147677</v>
+        <v>0</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="20">
@@ -1009,19 +1009,19 @@
         <v>575172642</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>0</v>
+        <v>575172642</v>
       </c>
       <c r="E20" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>0</v>
+        <v>575172642</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>-575172642</v>
+        <v>0</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="21">
@@ -1037,19 +1037,19 @@
         <v>61655471600</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>0</v>
+        <v>9467977800</v>
       </c>
       <c r="E21" s="3" t="n">
         <v>52187493800</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>52187493800</v>
+        <v>61655471600</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>-9467977800</v>
+        <v>0</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>84.64373468517918</v>
+        <v>100</v>
       </c>
     </row>
     <row r="22">
@@ -1065,19 +1065,19 @@
         <v>10654182000</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>0</v>
+        <v>10654182000</v>
       </c>
       <c r="E22" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>0</v>
+        <v>10654182000</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>-10654182000</v>
+        <v>0</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="23">
@@ -1093,19 +1093,19 @@
         <v>8063419229</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>0</v>
+        <v>8063419229</v>
       </c>
       <c r="E23" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>0</v>
+        <v>8063419229</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>-8063419229</v>
+        <v>0</v>
       </c>
       <c r="H23" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="24">
@@ -1121,19 +1121,19 @@
         <v>11668621099</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>0</v>
+        <v>11668621099</v>
       </c>
       <c r="E24" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>0</v>
+        <v>11668621099</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>-11668621099</v>
+        <v>0</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="25">
@@ -1149,19 +1149,19 @@
         <v>532966503</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>0</v>
+        <v>532966503</v>
       </c>
       <c r="E25" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>0</v>
+        <v>532966503</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>-532966503</v>
+        <v>0</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="26">
@@ -1177,19 +1177,19 @@
         <v>12076302500</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>0</v>
+        <v>11831302500</v>
       </c>
       <c r="E26" s="3" t="n">
         <v>245000000</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>245000000</v>
+        <v>12076302500</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>-11831302500</v>
+        <v>0</v>
       </c>
       <c r="H26" s="4" t="n">
-        <v>2.028766669268181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="27">
@@ -1205,19 +1205,19 @@
         <v>28552934680</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>0</v>
+        <v>28552934680</v>
       </c>
       <c r="E27" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>0</v>
+        <v>28552934680</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>-28552934680</v>
+        <v>0</v>
       </c>
       <c r="H27" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="28">
@@ -1233,19 +1233,19 @@
         <v>1858317230</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>0</v>
+        <v>1858317230</v>
       </c>
       <c r="E28" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>0</v>
+        <v>1858317230</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>-1858317230</v>
+        <v>0</v>
       </c>
       <c r="H28" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="29">
@@ -1261,19 +1261,19 @@
         <v>1417613763</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>0</v>
+        <v>1417613763</v>
       </c>
       <c r="E29" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>0</v>
+        <v>1417613763</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>-1417613763</v>
+        <v>0</v>
       </c>
       <c r="H29" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="30">
@@ -1289,19 +1289,19 @@
         <v>1292926000</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>0</v>
+        <v>1292926000</v>
       </c>
       <c r="E30" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>0</v>
+        <v>1292926000</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>-1292926000</v>
+        <v>0</v>
       </c>
       <c r="H30" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="31">
@@ -1317,19 +1317,19 @@
         <v>5257374241</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>0</v>
+        <v>5051110241</v>
       </c>
       <c r="E31" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>0</v>
+        <v>5051110241</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>-5257374241</v>
+        <v>-206264000</v>
       </c>
       <c r="H31" s="4" t="n">
-        <v>0</v>
+        <v>96.07667267832227</v>
       </c>
     </row>
     <row r="32">
@@ -1345,19 +1345,19 @@
         <v>4701405808</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>0</v>
+        <v>4606645808</v>
       </c>
       <c r="E32" s="3" t="n">
         <v>94760000</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>94760000</v>
+        <v>4701405808</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>-4606645808</v>
+        <v>0</v>
       </c>
       <c r="H32" s="4" t="n">
-        <v>2.015567340278404</v>
+        <v>100</v>
       </c>
     </row>
     <row r="33">
@@ -1373,19 +1373,19 @@
         <v>465249566</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>0</v>
+        <v>465249566</v>
       </c>
       <c r="E33" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>0</v>
+        <v>465249566</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>-465249566</v>
+        <v>0</v>
       </c>
       <c r="H33" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="34">
@@ -1401,19 +1401,19 @@
         <v>948269958</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>0</v>
+        <v>507369966</v>
       </c>
       <c r="E34" s="3" t="n">
         <v>440899992</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>440899992</v>
+        <v>948269958</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>-507369966</v>
+        <v>0</v>
       </c>
       <c r="H34" s="4" t="n">
-        <v>46.49519773144601</v>
+        <v>100</v>
       </c>
     </row>
     <row r="35">
@@ -1429,19 +1429,19 @@
         <v>943247000</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>0</v>
+        <v>774999698</v>
       </c>
       <c r="E35" s="3" t="n">
         <v>168247302</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>168247302</v>
+        <v>943247000</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>-774999698</v>
+        <v>0</v>
       </c>
       <c r="H35" s="4" t="n">
-        <v>17.83703547427132</v>
+        <v>100</v>
       </c>
     </row>
     <row r="36">
@@ -1457,19 +1457,19 @@
         <v>312595476</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>0</v>
+        <v>312595476</v>
       </c>
       <c r="E36" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>0</v>
+        <v>312595476</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>-312595476</v>
+        <v>0</v>
       </c>
       <c r="H36" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="37">
@@ -1485,19 +1485,19 @@
         <v>219851775</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>0</v>
+        <v>219851775</v>
       </c>
       <c r="E37" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>0</v>
+        <v>219851775</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>-219851775</v>
+        <v>0</v>
       </c>
       <c r="H37" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="38">
@@ -1905,19 +1905,19 @@
         <v>2405886712</v>
       </c>
       <c r="D52" s="3" t="n">
-        <v>0</v>
+        <v>2374286712</v>
       </c>
       <c r="E52" s="3" t="n">
         <v>31600000</v>
       </c>
       <c r="F52" s="3" t="n">
-        <v>31600000</v>
+        <v>2405886712</v>
       </c>
       <c r="G52" s="3" t="n">
-        <v>-2374286712</v>
+        <v>0</v>
       </c>
       <c r="H52" s="4" t="n">
-        <v>1.313445053018772</v>
+        <v>100</v>
       </c>
     </row>
     <row r="53">
@@ -2045,19 +2045,19 @@
         <v>1801912000</v>
       </c>
       <c r="D57" s="3" t="n">
-        <v>0</v>
+        <v>1780912000</v>
       </c>
       <c r="E57" s="3" t="n">
         <v>21000000</v>
       </c>
       <c r="F57" s="3" t="n">
-        <v>21000000</v>
+        <v>1801912000</v>
       </c>
       <c r="G57" s="3" t="n">
-        <v>-1780912000</v>
+        <v>0</v>
       </c>
       <c r="H57" s="4" t="n">
-        <v>1.165428722379339</v>
+        <v>100</v>
       </c>
     </row>
     <row r="58">
@@ -2073,19 +2073,19 @@
         <v>1367075285</v>
       </c>
       <c r="D58" s="3" t="n">
-        <v>0</v>
+        <v>721339185</v>
       </c>
       <c r="E58" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F58" s="3" t="n">
-        <v>0</v>
+        <v>721339185</v>
       </c>
       <c r="G58" s="3" t="n">
-        <v>-1367075285</v>
+        <v>-645736100</v>
       </c>
       <c r="H58" s="4" t="n">
-        <v>0</v>
+        <v>52.76513977794573</v>
       </c>
     </row>
     <row r="59">
@@ -2101,19 +2101,19 @@
         <v>338454320</v>
       </c>
       <c r="D59" s="3" t="n">
-        <v>0</v>
+        <v>338454320</v>
       </c>
       <c r="E59" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F59" s="3" t="n">
-        <v>0</v>
+        <v>338454320</v>
       </c>
       <c r="G59" s="3" t="n">
-        <v>-338454320</v>
+        <v>0</v>
       </c>
       <c r="H59" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="60">
@@ -2129,19 +2129,19 @@
         <v>887410440</v>
       </c>
       <c r="D60" s="3" t="n">
-        <v>0</v>
+        <v>887410440</v>
       </c>
       <c r="E60" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F60" s="3" t="n">
-        <v>0</v>
+        <v>887410440</v>
       </c>
       <c r="G60" s="3" t="n">
-        <v>-887410440</v>
+        <v>0</v>
       </c>
       <c r="H60" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="61">
@@ -2157,19 +2157,19 @@
         <v>1424797850</v>
       </c>
       <c r="D61" s="3" t="n">
-        <v>0</v>
+        <v>212772837</v>
       </c>
       <c r="E61" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F61" s="3" t="n">
-        <v>0</v>
+        <v>212772837</v>
       </c>
       <c r="G61" s="3" t="n">
-        <v>-1424797850</v>
+        <v>-1212025013</v>
       </c>
       <c r="H61" s="4" t="n">
-        <v>0</v>
+        <v>14.93354562543732</v>
       </c>
     </row>
     <row r="62">
@@ -2185,19 +2185,19 @@
         <v>1117262389</v>
       </c>
       <c r="D62" s="3" t="n">
-        <v>0</v>
+        <v>1116362329</v>
       </c>
       <c r="E62" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F62" s="3" t="n">
-        <v>0</v>
+        <v>1116362329</v>
       </c>
       <c r="G62" s="3" t="n">
-        <v>-1117262389</v>
+        <v>-900060</v>
       </c>
       <c r="H62" s="4" t="n">
-        <v>0</v>
+        <v>99.91944058899132</v>
       </c>
     </row>
     <row r="63">
@@ -2213,19 +2213,19 @@
         <v>509262312</v>
       </c>
       <c r="D63" s="3" t="n">
-        <v>0</v>
+        <v>509262312</v>
       </c>
       <c r="E63" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F63" s="3" t="n">
-        <v>0</v>
+        <v>509262312</v>
       </c>
       <c r="G63" s="3" t="n">
-        <v>-509262312</v>
+        <v>0</v>
       </c>
       <c r="H63" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="64">
@@ -2241,19 +2241,19 @@
         <v>373421530</v>
       </c>
       <c r="D64" s="3" t="n">
-        <v>0</v>
+        <v>373421530</v>
       </c>
       <c r="E64" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F64" s="3" t="n">
-        <v>0</v>
+        <v>373421530</v>
       </c>
       <c r="G64" s="3" t="n">
-        <v>-373421530</v>
+        <v>0</v>
       </c>
       <c r="H64" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="65">
@@ -2269,19 +2269,19 @@
         <v>552591787</v>
       </c>
       <c r="D65" s="3" t="n">
-        <v>0</v>
+        <v>552591787</v>
       </c>
       <c r="E65" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F65" s="3" t="n">
-        <v>0</v>
+        <v>552591787</v>
       </c>
       <c r="G65" s="3" t="n">
-        <v>-552591787</v>
+        <v>0</v>
       </c>
       <c r="H65" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="66">
@@ -2297,19 +2297,19 @@
         <v>735655752</v>
       </c>
       <c r="D66" s="3" t="n">
-        <v>0</v>
+        <v>541055752</v>
       </c>
       <c r="E66" s="3" t="n">
         <v>194600000</v>
       </c>
       <c r="F66" s="3" t="n">
-        <v>194600000</v>
+        <v>735655752</v>
       </c>
       <c r="G66" s="3" t="n">
-        <v>-541055752</v>
+        <v>0</v>
       </c>
       <c r="H66" s="4" t="n">
-        <v>26.45259001522767</v>
+        <v>100</v>
       </c>
     </row>
     <row r="67">
@@ -2325,19 +2325,19 @@
         <v>289499767</v>
       </c>
       <c r="D67" s="3" t="n">
-        <v>0</v>
+        <v>289499767</v>
       </c>
       <c r="E67" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F67" s="3" t="n">
-        <v>0</v>
+        <v>289499767</v>
       </c>
       <c r="G67" s="3" t="n">
-        <v>-289499767</v>
+        <v>0</v>
       </c>
       <c r="H67" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="68">
@@ -2353,19 +2353,19 @@
         <v>429267455</v>
       </c>
       <c r="D68" s="3" t="n">
-        <v>0</v>
+        <v>429267455</v>
       </c>
       <c r="E68" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F68" s="3" t="n">
-        <v>0</v>
+        <v>429267455</v>
       </c>
       <c r="G68" s="3" t="n">
-        <v>-429267455</v>
+        <v>0</v>
       </c>
       <c r="H68" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="69">
@@ -2381,19 +2381,19 @@
         <v>153251633</v>
       </c>
       <c r="D69" s="3" t="n">
-        <v>0</v>
+        <v>153251633</v>
       </c>
       <c r="E69" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F69" s="3" t="n">
-        <v>0</v>
+        <v>153251633</v>
       </c>
       <c r="G69" s="3" t="n">
-        <v>-153251633</v>
+        <v>0</v>
       </c>
       <c r="H69" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="70">
@@ -2409,19 +2409,19 @@
         <v>329330796</v>
       </c>
       <c r="D70" s="3" t="n">
-        <v>0</v>
+        <v>329330796</v>
       </c>
       <c r="E70" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F70" s="3" t="n">
-        <v>0</v>
+        <v>329330796</v>
       </c>
       <c r="G70" s="3" t="n">
-        <v>-329330796</v>
+        <v>0</v>
       </c>
       <c r="H70" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="71">
@@ -2437,19 +2437,19 @@
         <v>270659900</v>
       </c>
       <c r="D71" s="3" t="n">
-        <v>0</v>
+        <v>270659900</v>
       </c>
       <c r="E71" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F71" s="3" t="n">
-        <v>0</v>
+        <v>270659900</v>
       </c>
       <c r="G71" s="3" t="n">
-        <v>-270659900</v>
+        <v>0</v>
       </c>
       <c r="H71" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="72">
@@ -2465,19 +2465,19 @@
         <v>654395500</v>
       </c>
       <c r="D72" s="3" t="n">
-        <v>0</v>
+        <v>654395500</v>
       </c>
       <c r="E72" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F72" s="3" t="n">
-        <v>0</v>
+        <v>654395500</v>
       </c>
       <c r="G72" s="3" t="n">
-        <v>-654395500</v>
+        <v>0</v>
       </c>
       <c r="H72" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="73">
@@ -2493,19 +2493,19 @@
         <v>448879549</v>
       </c>
       <c r="D73" s="3" t="n">
-        <v>0</v>
+        <v>448879549</v>
       </c>
       <c r="E73" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F73" s="3" t="n">
-        <v>0</v>
+        <v>448879549</v>
       </c>
       <c r="G73" s="3" t="n">
-        <v>-448879549</v>
+        <v>0</v>
       </c>
       <c r="H73" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="74">
@@ -2521,19 +2521,19 @@
         <v>1291889268</v>
       </c>
       <c r="D74" s="3" t="n">
-        <v>0</v>
+        <v>350390301</v>
       </c>
       <c r="E74" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F74" s="3" t="n">
-        <v>0</v>
+        <v>350390301</v>
       </c>
       <c r="G74" s="3" t="n">
-        <v>-1291889268</v>
+        <v>-941498967</v>
       </c>
       <c r="H74" s="4" t="n">
-        <v>0</v>
+        <v>27.12231687956092</v>
       </c>
     </row>
     <row r="75">
@@ -2577,19 +2577,19 @@
         <v>992988041</v>
       </c>
       <c r="D76" s="3" t="n">
-        <v>0</v>
+        <v>992988041</v>
       </c>
       <c r="E76" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F76" s="3" t="n">
-        <v>0</v>
+        <v>992988041</v>
       </c>
       <c r="G76" s="3" t="n">
-        <v>-992988041</v>
+        <v>0</v>
       </c>
       <c r="H76" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="77">
@@ -2605,19 +2605,19 @@
         <v>85061928740</v>
       </c>
       <c r="D77" s="3" t="n">
-        <v>0</v>
+        <v>85061928740</v>
       </c>
       <c r="E77" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F77" s="3" t="n">
-        <v>0</v>
+        <v>85061928740</v>
       </c>
       <c r="G77" s="3" t="n">
-        <v>-85061928740</v>
+        <v>0</v>
       </c>
       <c r="H77" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="78">
@@ -2633,19 +2633,19 @@
         <v>1028700867</v>
       </c>
       <c r="D78" s="3" t="n">
-        <v>0</v>
+        <v>1028700867</v>
       </c>
       <c r="E78" s="3" t="n">
         <v>0</v>
       </c>
       <c r="F78" s="3" t="n">
-        <v>0</v>
+        <v>1028700867</v>
       </c>
       <c r="G78" s="3" t="n">
-        <v>-1028700867</v>
+        <v>0</v>
       </c>
       <c r="H78" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="79">
@@ -2661,19 +2661,19 @@
         <v>8905641688</v>
       </c>
       <c r="D79" s="3" t="n">
-        <v>0</v>
+        <v>8755641688</v>
       </c>
       <c r="E79" s="3" t="n">
         <v>150000000</v>
       </c>
       <c r="F79" s="3" t="n">
-        <v>150000000</v>
+        <v>8905641688</v>
       </c>
       <c r="G79" s="3" t="n">
-        <v>-8755641688</v>
+        <v>0</v>
       </c>
       <c r="H79" s="4" t="n">
-        <v>1.684325568612524</v>
+        <v>100</v>
       </c>
     </row>
     <row r="80">
@@ -2689,19 +2689,19 @@
         <v>11974816559</v>
       </c>
       <c r="D80" s="3" t="n">
-        <v>0</v>
+        <v>11799027759</v>
       </c>
       <c r="E80" s="3" t="n">
         <v>175788800</v>
       </c>
       <c r="F80" s="3" t="n">
-        <v>175788800</v>
+        <v>11974816559</v>
       </c>
       <c r="G80" s="3" t="n">
-        <v>-11799027759</v>
+        <v>0</v>
       </c>
       <c r="H80" s="4" t="n">
-        <v>1.467987414536894</v>
+        <v>100</v>
       </c>
     </row>
     <row r="81">

</xml_diff>